<commit_message>
Added new RDF data schemes and visual schemes for economy-table101-105, fixed XLSX spreadsheets for economy-table101-104
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table101.xlsx
+++ b/sources/table_normalization/xlsx/economy-table101.xlsx
@@ -279,7 +279,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -332,10 +332,13 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Гиперссылка" xfId="2" builtinId="8"/>
@@ -343,34 +346,6 @@
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -453,6 +428,34 @@
         <color auto="1"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -467,16 +470,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="table_3a_bankruptcies_england_wales_sa" displayName="table_3a_bankruptcies_england_wales_sa" ref="A6:H61" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="table_3a_bankruptcies_england_wales_sa" displayName="table_3a_bankruptcies_england_wales_sa" ref="A6:H61" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <tableColumns count="8">
-    <tableColumn id="1" name="Year" dataDxfId="9"/>
-    <tableColumn id="2" name="Quarter" dataDxfId="8"/>
-    <tableColumn id="3" name="Total bankruptcies [note 8]" dataDxfId="7"/>
-    <tableColumn id="4" name="r_total_bankruptcies" dataDxfId="6"/>
-    <tableColumn id="5" name="Creditors' petitions [note 2]" dataDxfId="5"/>
-    <tableColumn id="6" name="r_creditor" dataDxfId="4"/>
-    <tableColumn id="7" name="Debtors' applications [note 3]" dataDxfId="3"/>
-    <tableColumn id="8" name="r_debtor" dataDxfId="2"/>
+    <tableColumn id="1" name="Year" dataDxfId="7"/>
+    <tableColumn id="2" name="Quarter" dataDxfId="6"/>
+    <tableColumn id="3" name="Total bankruptcies [note 8]" dataDxfId="5"/>
+    <tableColumn id="4" name="r_total_bankruptcies" dataDxfId="4"/>
+    <tableColumn id="5" name="Creditors' petitions [note 2]" dataDxfId="3"/>
+    <tableColumn id="6" name="r_creditor" dataDxfId="2"/>
+    <tableColumn id="7" name="Debtors' applications [note 3]" dataDxfId="1"/>
+    <tableColumn id="8" name="r_debtor" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="none" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -833,7 +836,7 @@
       <c r="M3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="36" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="6"/>
@@ -873,19 +876,19 @@
       <c r="B6" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="40" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="E6" s="40" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="34" t="s">
+      <c r="G6" s="40" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="35" t="s">
@@ -2239,16 +2242,16 @@
       <c r="H58" s="13"/>
     </row>
     <row r="59" spans="1:9" ht="12.65" customHeight="1">
-      <c r="A59" s="39" t="s">
+      <c r="A59" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B59" s="36"/>
-      <c r="C59" s="37"/>
-      <c r="D59" s="37"/>
-      <c r="E59" s="36"/>
-      <c r="F59" s="36"/>
-      <c r="G59" s="36"/>
-      <c r="H59" s="36"/>
+      <c r="B59" s="38"/>
+      <c r="C59" s="39"/>
+      <c r="D59" s="39"/>
+      <c r="E59" s="38"/>
+      <c r="F59" s="38"/>
+      <c r="G59" s="38"/>
+      <c r="H59" s="38"/>
     </row>
     <row r="60" spans="1:9" ht="15" customHeight="1">
       <c r="A60" s="17" t="s">

</xml_diff>